<commit_message>
Datos de Venta Nueva actualizados + % de crecimiento por barra
- Datos: VN 2026 actualizada ($6,339,644 -> $6,962,163).
- Gráfica "Por área": cada barra muestra su % de crecimiento
  (2025 vs 2024, PTO vs 2025, Real vs 2025 mismo periodo).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EXCEL/Town Hall Julio 2026.xlsx
+++ b/EXCEL/Town Hall Julio 2026.xlsx
@@ -12,7 +12,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="31">
+  <si>
+    <t>Venta Nueva 2024</t>
+  </si>
   <si>
     <t>AREA</t>
   </si>
@@ -68,10 +71,10 @@
     <t>BENEFICIOS</t>
   </si>
   <si>
-    <t>BONO</t>
+    <t>DAÑOS</t>
   </si>
   <si>
-    <t>DAÑOS</t>
+    <t>BONO</t>
   </si>
   <si>
     <t>INTERNACIONAL</t>
@@ -86,28 +89,22 @@
     <t>LP</t>
   </si>
   <si>
+    <t>Venta Nueva 2025</t>
+  </si>
+  <si>
     <t>2026 Real</t>
+  </si>
+  <si>
+    <t>Venta Nueva 2026</t>
+  </si>
+  <si>
+    <t>Venta Nueva PTO 2026</t>
   </si>
   <si>
     <t>PTO 2026</t>
   </si>
   <si>
     <t>ÁREA</t>
-  </si>
-  <si>
-    <t>HONORARIOS</t>
-  </si>
-  <si>
-    <t>Venta Nueva 2024</t>
-  </si>
-  <si>
-    <t>Venta Nueva 2025</t>
-  </si>
-  <si>
-    <t>Venta Nueva 2026</t>
-  </si>
-  <si>
-    <t>Venta Nueva PTO 2026</t>
   </si>
 </sst>
 </file>
@@ -204,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -226,6 +223,8 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="3" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="10" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -470,51 +469,51 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="5">
@@ -557,7 +556,7 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B4" s="5">
         <v>513.0</v>
@@ -602,7 +601,7 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B5" s="5">
         <v>138677.0</v>
@@ -647,7 +646,7 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B6" s="5">
         <v>2501929.0</v>
@@ -692,7 +691,7 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B7" s="5">
         <v>452640.0</v>
@@ -782,7 +781,7 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -807,7 +806,7 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B10" s="5">
         <v>1355603.0</v>
@@ -852,7 +851,7 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11" s="5">
         <v>439480.0</v>
@@ -897,7 +896,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B12" s="5">
         <v>429530.0</v>
@@ -942,7 +941,7 @@
     </row>
     <row r="13">
       <c r="A13" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B13" s="7">
         <f t="shared" ref="B13:N13" si="2">SUM(B3:B12)</f>
@@ -1049,51 +1048,51 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L17" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M17" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N17" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -1114,26 +1113,14 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19" s="5">
-        <v>35106.0</v>
-      </c>
-      <c r="C19" s="5">
-        <v>10234.0</v>
-      </c>
-      <c r="D19" s="5">
-        <v>23167.0</v>
-      </c>
-      <c r="E19" s="5">
-        <v>26615.0</v>
-      </c>
-      <c r="F19" s="5">
-        <v>54185.0</v>
-      </c>
-      <c r="G19" s="5">
-        <v>6999.0</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
       <c r="H19" s="5">
         <v>15170.0</v>
       </c>
@@ -1152,12 +1139,12 @@
       <c r="M19" s="6"/>
       <c r="N19" s="5">
         <f t="shared" si="3"/>
-        <v>207651</v>
+        <v>51345</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B20" s="5">
         <v>155220.0</v>
@@ -1199,10 +1186,14 @@
         <f t="shared" si="3"/>
         <v>8699280</v>
       </c>
+      <c r="P20" s="8">
+        <f>SUM(B28:G28)</f>
+        <v>67362388</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B21" s="5">
         <v>2101265.0</v>
@@ -1244,10 +1235,14 @@
         <f t="shared" si="3"/>
         <v>49916203</v>
       </c>
+      <c r="P21" s="9">
+        <f>(N43/P20)-1</f>
+        <v>0.222507477</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B22" s="5">
         <v>1123541.0</v>
@@ -1337,7 +1332,7 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -1358,7 +1353,7 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B25" s="5">
         <v>1647297.0</v>
@@ -1403,7 +1398,7 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B26" s="5">
         <v>739024.0</v>
@@ -1448,7 +1443,7 @@
     </row>
     <row r="27">
       <c r="A27" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B27" s="5">
         <v>539098.0</v>
@@ -1493,31 +1488,31 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B28" s="7">
         <f t="shared" ref="B28:N28" si="4">SUM(B19:B27)</f>
-        <v>8357281</v>
+        <v>8322175</v>
       </c>
       <c r="C28" s="7">
         <f t="shared" si="4"/>
-        <v>12293428</v>
+        <v>12283194</v>
       </c>
       <c r="D28" s="7">
         <f t="shared" si="4"/>
-        <v>11324240</v>
+        <v>11301073</v>
       </c>
       <c r="E28" s="7">
         <f t="shared" si="4"/>
-        <v>12577085</v>
+        <v>12550470</v>
       </c>
       <c r="F28" s="7">
         <f t="shared" si="4"/>
-        <v>10500730</v>
+        <v>10446545</v>
       </c>
       <c r="G28" s="7">
         <f t="shared" si="4"/>
-        <v>12465930</v>
+        <v>12458931</v>
       </c>
       <c r="H28" s="7">
         <f t="shared" si="4"/>
@@ -1545,7 +1540,7 @@
       </c>
       <c r="N28" s="7">
         <f t="shared" si="4"/>
-        <v>147392892</v>
+        <v>147236586</v>
       </c>
     </row>
     <row r="29">
@@ -1582,7 +1577,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -1600,51 +1595,51 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K32" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L32" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M32" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N32" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B33" s="6">
         <v>0.0</v>
@@ -1677,7 +1672,7 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B34" s="5">
         <v>14753.0</v>
@@ -1710,7 +1705,7 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B35" s="5">
         <v>603090.0</v>
@@ -1743,7 +1738,7 @@
     </row>
     <row r="36">
       <c r="A36" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B36" s="5">
         <v>3394150.0</v>
@@ -1776,7 +1771,7 @@
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B37" s="5">
         <v>7877374.0</v>
@@ -1842,7 +1837,7 @@
     </row>
     <row r="39">
       <c r="A39" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B39" s="6">
         <v>0.0</v>
@@ -1875,7 +1870,7 @@
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B40" s="5">
         <v>2324944.0</v>
@@ -1908,7 +1903,7 @@
     </row>
     <row r="41">
       <c r="A41" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B41" s="5">
         <v>246530.0</v>
@@ -1941,7 +1936,7 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B42" s="5">
         <v>597336.0</v>
@@ -1974,7 +1969,7 @@
     </row>
     <row r="43">
       <c r="A43" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B43" s="7">
         <f t="shared" ref="B43:N43" si="6">SUM(B34:B42)</f>
@@ -2063,7 +2058,7 @@
     </row>
     <row r="46">
       <c r="A46" s="1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -2081,51 +2076,51 @@
     </row>
     <row r="47">
       <c r="A47" s="4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K47" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L47" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M47" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N47" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B48" s="5">
         <v>39216.0</v>
@@ -2169,7 +2164,7 @@
     </row>
     <row r="49">
       <c r="A49" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B49" s="5">
         <v>349322.97</v>
@@ -2213,43 +2208,43 @@
     </row>
     <row r="50">
       <c r="A50" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B50" s="5">
-        <v>1349905.28</v>
-      </c>
-      <c r="C50" s="5">
-        <v>5125956.08</v>
-      </c>
-      <c r="D50" s="5">
-        <v>6970194.25</v>
-      </c>
-      <c r="E50" s="5">
-        <v>4489335.51</v>
-      </c>
-      <c r="F50" s="5">
-        <v>3559102.06</v>
-      </c>
-      <c r="G50" s="5">
-        <v>4832733.74</v>
-      </c>
-      <c r="H50" s="5">
-        <v>3710266.03</v>
-      </c>
-      <c r="I50" s="5">
-        <v>2497612.59</v>
-      </c>
-      <c r="J50" s="5">
-        <v>3828285.91</v>
-      </c>
-      <c r="K50" s="5">
-        <v>2216879.52</v>
-      </c>
-      <c r="L50" s="5">
-        <v>9877816.33</v>
-      </c>
-      <c r="M50" s="5">
-        <v>1.614518025E7</v>
+        <v>18</v>
+      </c>
+      <c r="B50" s="6">
+        <v>1428965.84</v>
+      </c>
+      <c r="C50" s="6">
+        <v>5205016.64</v>
+      </c>
+      <c r="D50" s="6">
+        <v>7049254.81</v>
+      </c>
+      <c r="E50" s="6">
+        <v>4568396.069999999</v>
+      </c>
+      <c r="F50" s="6">
+        <v>3638162.62</v>
+      </c>
+      <c r="G50" s="6">
+        <v>4911794.3</v>
+      </c>
+      <c r="H50" s="6">
+        <v>3789326.59</v>
+      </c>
+      <c r="I50" s="6">
+        <v>2576673.15</v>
+      </c>
+      <c r="J50" s="6">
+        <v>3907346.47</v>
+      </c>
+      <c r="K50" s="6">
+        <v>2295940.08</v>
+      </c>
+      <c r="L50" s="6">
+        <v>9956876.89</v>
+      </c>
+      <c r="M50" s="6">
+        <v>1.622424081E7</v>
       </c>
       <c r="N50" s="5">
         <v>6.460326755E7</v>
@@ -2257,7 +2252,7 @@
     </row>
     <row r="51">
       <c r="A51" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B51" s="5">
         <v>7715758.0</v>
@@ -2343,242 +2338,210 @@
     </row>
     <row r="53">
       <c r="A53" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B53" s="5">
-        <v>79060.56</v>
-      </c>
-      <c r="C53" s="5">
-        <v>79060.56</v>
-      </c>
-      <c r="D53" s="5">
-        <v>79060.56</v>
-      </c>
-      <c r="E53" s="5">
-        <v>79060.56</v>
-      </c>
-      <c r="F53" s="5">
-        <v>79060.56</v>
-      </c>
-      <c r="G53" s="5">
-        <v>79060.56</v>
-      </c>
-      <c r="H53" s="5">
-        <v>79060.56</v>
-      </c>
-      <c r="I53" s="5">
-        <v>79060.56</v>
-      </c>
-      <c r="J53" s="5">
-        <v>79060.56</v>
-      </c>
-      <c r="K53" s="5">
-        <v>79060.56</v>
-      </c>
-      <c r="L53" s="5">
-        <v>79060.56</v>
-      </c>
-      <c r="M53" s="5">
-        <v>79060.56</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="B53" s="6"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="6"/>
+      <c r="E53" s="6"/>
+      <c r="F53" s="6"/>
+      <c r="G53" s="6"/>
+      <c r="H53" s="6"/>
+      <c r="I53" s="6"/>
+      <c r="J53" s="6"/>
+      <c r="K53" s="6"/>
+      <c r="L53" s="6"/>
+      <c r="M53" s="6"/>
       <c r="N53" s="5">
-        <v>948726.72</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B54" s="6"/>
-      <c r="C54" s="6"/>
-      <c r="D54" s="6"/>
-      <c r="E54" s="6"/>
-      <c r="F54" s="6"/>
-      <c r="G54" s="6"/>
-      <c r="H54" s="6"/>
-      <c r="I54" s="6"/>
-      <c r="J54" s="6"/>
-      <c r="K54" s="6"/>
-      <c r="L54" s="6"/>
-      <c r="M54" s="6"/>
+        <v>22</v>
+      </c>
+      <c r="B54" s="5">
+        <v>2247297.0</v>
+      </c>
+      <c r="C54" s="5">
+        <v>1516629.0</v>
+      </c>
+      <c r="D54" s="5">
+        <v>2109261.0</v>
+      </c>
+      <c r="E54" s="5">
+        <v>2736368.0</v>
+      </c>
+      <c r="F54" s="5">
+        <v>1780201.0</v>
+      </c>
+      <c r="G54" s="5">
+        <v>4289063.0</v>
+      </c>
+      <c r="H54" s="5">
+        <v>2842164.0</v>
+      </c>
+      <c r="I54" s="5">
+        <v>1649901.0</v>
+      </c>
+      <c r="J54" s="5">
+        <v>3149060.0</v>
+      </c>
+      <c r="K54" s="5">
+        <v>2544478.0</v>
+      </c>
+      <c r="L54" s="5">
+        <v>2101675.0</v>
+      </c>
+      <c r="M54" s="5">
+        <v>1654422.0</v>
+      </c>
       <c r="N54" s="5">
-        <v>0.0</v>
+        <v>2.8620519E7</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B55" s="5">
-        <v>2247297.0</v>
+        <v>1955690.99</v>
       </c>
       <c r="C55" s="5">
-        <v>1516629.0</v>
+        <v>3728707.74</v>
       </c>
       <c r="D55" s="5">
-        <v>2109261.0</v>
+        <v>2588312.73</v>
       </c>
       <c r="E55" s="5">
-        <v>2736368.0</v>
+        <v>4848590.83</v>
       </c>
       <c r="F55" s="5">
-        <v>1780201.0</v>
+        <v>6041959.38</v>
       </c>
       <c r="G55" s="5">
-        <v>4289063.0</v>
+        <v>1362692.18</v>
       </c>
       <c r="H55" s="5">
-        <v>2842164.0</v>
+        <v>5263250.98</v>
       </c>
       <c r="I55" s="5">
-        <v>1649901.0</v>
+        <v>7835926.84</v>
       </c>
       <c r="J55" s="5">
-        <v>3149060.0</v>
+        <v>2092612.01</v>
       </c>
       <c r="K55" s="5">
-        <v>2544478.0</v>
+        <v>1724700.9</v>
       </c>
       <c r="L55" s="5">
-        <v>2101675.0</v>
+        <v>1812339.0</v>
       </c>
       <c r="M55" s="5">
-        <v>1654422.0</v>
+        <v>1878158.5</v>
       </c>
       <c r="N55" s="5">
-        <v>2.8620519E7</v>
+        <v>4.113294208E7</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B56" s="5">
-        <v>1955690.99</v>
+        <v>1209284.07</v>
       </c>
       <c r="C56" s="5">
-        <v>3728707.74</v>
+        <v>1068369.31</v>
       </c>
       <c r="D56" s="5">
-        <v>2588312.73</v>
+        <v>1423036.29</v>
       </c>
       <c r="E56" s="5">
-        <v>4848590.83</v>
+        <v>1418879.06</v>
       </c>
       <c r="F56" s="5">
-        <v>6041959.38</v>
+        <v>1272439.89</v>
       </c>
       <c r="G56" s="5">
-        <v>1362692.18</v>
+        <v>1007451.93</v>
       </c>
       <c r="H56" s="5">
-        <v>5263250.98</v>
+        <v>1681263.31</v>
       </c>
       <c r="I56" s="5">
-        <v>7835926.84</v>
+        <v>897767.59</v>
       </c>
       <c r="J56" s="5">
-        <v>2092612.01</v>
+        <v>1689005.27</v>
       </c>
       <c r="K56" s="5">
-        <v>1724700.9</v>
+        <v>1765675.14</v>
       </c>
       <c r="L56" s="5">
-        <v>1812339.0</v>
+        <v>1361205.8</v>
       </c>
       <c r="M56" s="5">
-        <v>1878158.5</v>
+        <v>1162598.39</v>
       </c>
       <c r="N56" s="5">
-        <v>4.113294208E7</v>
+        <v>1.595697605E7</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B57" s="5">
-        <v>1209284.07</v>
-      </c>
-      <c r="C57" s="5">
-        <v>1068369.31</v>
-      </c>
-      <c r="D57" s="5">
-        <v>1423036.29</v>
-      </c>
-      <c r="E57" s="5">
-        <v>1418879.06</v>
-      </c>
-      <c r="F57" s="5">
-        <v>1272439.89</v>
-      </c>
-      <c r="G57" s="5">
-        <v>1007451.93</v>
-      </c>
-      <c r="H57" s="5">
-        <v>1681263.31</v>
-      </c>
-      <c r="I57" s="5">
-        <v>897767.59</v>
-      </c>
-      <c r="J57" s="5">
-        <v>1689005.27</v>
-      </c>
-      <c r="K57" s="5">
-        <v>1765675.14</v>
-      </c>
-      <c r="L57" s="5">
-        <v>1361205.8</v>
-      </c>
-      <c r="M57" s="5">
-        <v>1162598.39</v>
-      </c>
-      <c r="N57" s="5">
-        <v>1.595697605E7</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B58" s="7">
+      <c r="A57" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B57" s="7">
         <v>1.716225547E7</v>
       </c>
-      <c r="C58" s="7">
+      <c r="C57" s="7">
         <v>1.652216094E7</v>
       </c>
-      <c r="D58" s="7">
+      <c r="D57" s="7">
         <v>1.819792195E7</v>
       </c>
-      <c r="E58" s="7">
+      <c r="E57" s="7">
         <v>1.819793085E7</v>
       </c>
-      <c r="F58" s="7">
+      <c r="F57" s="7">
         <v>1.6962334E7</v>
       </c>
-      <c r="G58" s="7">
+      <c r="G57" s="7">
         <v>1.684499886E7</v>
       </c>
-      <c r="H58" s="7">
+      <c r="H57" s="7">
         <v>1.800243126E7</v>
       </c>
-      <c r="I58" s="7">
+      <c r="I57" s="7">
         <v>1.79395137E7</v>
       </c>
-      <c r="J58" s="7">
+      <c r="J57" s="7">
         <v>1.8349415E7</v>
       </c>
-      <c r="K58" s="7">
+      <c r="K57" s="7">
         <v>1.42717742E7</v>
       </c>
-      <c r="L58" s="7">
+      <c r="L57" s="7">
         <v>2.041676494E7</v>
       </c>
-      <c r="M58" s="7">
+      <c r="M57" s="7">
         <v>2.954457327E7</v>
       </c>
-      <c r="N58" s="7">
+      <c r="N57" s="7">
         <v>2.2241207444E8</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="H62" s="8">
+        <f>N57</f>
+        <v>222412074.4</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="H63" s="10">
+        <f>N43/H62</f>
+        <v>0.3702632746</v>
       </c>
     </row>
   </sheetData>
@@ -2604,7 +2567,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2622,51 +2585,51 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -2687,7 +2650,7 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -2716,7 +2679,7 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -2784,7 +2747,7 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -2807,7 +2770,7 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" s="5">
         <v>596434.0</v>
@@ -2852,7 +2815,7 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="5">
@@ -2885,7 +2848,7 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -2906,7 +2869,7 @@
     </row>
     <row r="11">
       <c r="A11" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B11" s="7">
         <f t="shared" ref="B11:N11" si="2">SUM(B3:B10)</f>
@@ -2995,7 +2958,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -3013,51 +2976,51 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L15" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M15" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N15" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -3078,7 +3041,7 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B17" s="5">
         <v>12811.0</v>
@@ -3117,7 +3080,7 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="5">
@@ -3201,7 +3164,7 @@
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -3222,7 +3185,7 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B21" s="5">
         <v>291693.0</v>
@@ -3264,10 +3227,14 @@
         <f t="shared" si="3"/>
         <v>6234087</v>
       </c>
+      <c r="P21" s="9">
+        <f>(N24/N11)-1</f>
+        <v>0.5423563792</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="5">
@@ -3310,7 +3277,7 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B23" s="5">
         <v>3124.0</v>
@@ -3355,7 +3322,7 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B24" s="7">
         <f t="shared" ref="B24:N24" si="4">SUM(B16:B23)</f>
@@ -3408,6 +3375,10 @@
       <c r="N24" s="7">
         <f t="shared" si="4"/>
         <v>21287612</v>
+      </c>
+      <c r="P24" s="8">
+        <f>SUM(B24:G24)</f>
+        <v>9355878</v>
       </c>
     </row>
     <row r="25">
@@ -3425,6 +3396,10 @@
       <c r="L25" s="8"/>
       <c r="M25" s="8"/>
       <c r="N25" s="8"/>
+      <c r="P25" s="10">
+        <f>(N36/P24)-1</f>
+        <v>-0.2558514551</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8"/>
@@ -3444,7 +3419,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -3462,51 +3437,51 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K28" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L28" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M28" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N28" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B29" s="5">
         <v>0.0</v>
@@ -3523,7 +3498,9 @@
       <c r="F29" s="5">
         <v>0.0</v>
       </c>
-      <c r="G29" s="6"/>
+      <c r="G29" s="5">
+        <v>0.0</v>
+      </c>
       <c r="H29" s="6"/>
       <c r="I29" s="6"/>
       <c r="J29" s="6"/>
@@ -3537,7 +3514,7 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B30" s="5">
         <v>4319.0</v>
@@ -3570,19 +3547,19 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B31" s="5">
         <v>156691.0</v>
       </c>
       <c r="C31" s="5">
-        <v>2864479.0</v>
+        <v>2335708.0</v>
       </c>
       <c r="D31" s="5">
-        <v>183020.0</v>
+        <v>173018.0</v>
       </c>
       <c r="E31" s="5">
-        <v>474025.0</v>
+        <v>346255.0</v>
       </c>
       <c r="F31" s="5">
         <v>474088.0</v>
@@ -3598,7 +3575,7 @@
       <c r="M31" s="6"/>
       <c r="N31" s="5">
         <f t="shared" si="5"/>
-        <v>4251092</v>
+        <v>3584549</v>
       </c>
     </row>
     <row r="32">
@@ -3621,7 +3598,7 @@
         <v>138129.0</v>
       </c>
       <c r="G32" s="5">
-        <v>328801.0</v>
+        <v>1639698.0</v>
       </c>
       <c r="H32" s="6"/>
       <c r="I32" s="6"/>
@@ -3631,12 +3608,12 @@
       <c r="M32" s="6"/>
       <c r="N32" s="5">
         <f t="shared" si="5"/>
-        <v>1072389</v>
+        <v>2383286</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B33" s="5">
         <v>677647.0</v>
@@ -3669,7 +3646,7 @@
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B34" s="5">
         <v>95738.0</v>
@@ -3686,7 +3663,9 @@
       <c r="F34" s="5">
         <v>0.0</v>
       </c>
-      <c r="G34" s="6"/>
+      <c r="G34" s="5">
+        <v>0.0</v>
+      </c>
       <c r="H34" s="6"/>
       <c r="I34" s="6"/>
       <c r="J34" s="6"/>
@@ -3700,7 +3679,7 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B35" s="5">
         <v>44101.0</v>
@@ -3709,16 +3688,16 @@
         <v>72940.0</v>
       </c>
       <c r="D35" s="5">
-        <v>108033.0</v>
+        <v>103426.0</v>
       </c>
       <c r="E35" s="5">
         <v>75419.0</v>
       </c>
       <c r="F35" s="5">
-        <v>67343.0</v>
+        <v>66426.0</v>
       </c>
       <c r="G35" s="5">
-        <v>114812.0</v>
+        <v>98501.0</v>
       </c>
       <c r="H35" s="6"/>
       <c r="I35" s="6"/>
@@ -3728,12 +3707,12 @@
       <c r="M35" s="6"/>
       <c r="N35" s="5">
         <f t="shared" si="5"/>
-        <v>482648</v>
+        <v>460813</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B36" s="7">
         <f t="shared" ref="B36:N36" si="6">SUM(B29:B35)</f>
@@ -3741,23 +3720,23 @@
       </c>
       <c r="C36" s="7">
         <f t="shared" si="6"/>
-        <v>5188116</v>
+        <v>4659345</v>
       </c>
       <c r="D36" s="7">
         <f t="shared" si="6"/>
-        <v>262694</v>
+        <v>248085</v>
       </c>
       <c r="E36" s="7">
         <f t="shared" si="6"/>
-        <v>621855</v>
+        <v>494085</v>
       </c>
       <c r="F36" s="7">
         <f t="shared" si="6"/>
-        <v>517492</v>
+        <v>516575</v>
       </c>
       <c r="G36" s="7">
         <f t="shared" si="6"/>
-        <v>-1361921</v>
+        <v>-67335</v>
       </c>
       <c r="H36" s="7">
         <f t="shared" si="6"/>
@@ -3785,7 +3764,7 @@
       </c>
       <c r="N36" s="7">
         <f t="shared" si="6"/>
-        <v>6339644</v>
+        <v>6962163</v>
       </c>
     </row>
     <row r="37">
@@ -3822,7 +3801,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -3840,51 +3819,51 @@
     </row>
     <row r="40">
       <c r="A40" s="4" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K40" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L40" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M40" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N40" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B41" s="5">
         <v>39216.0</v>
@@ -3927,7 +3906,7 @@
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B42" s="5">
         <v>200000.0</v>
@@ -3972,7 +3951,7 @@
     </row>
     <row r="43">
       <c r="A43" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B43" s="5">
         <v>200000.0</v>
@@ -4062,7 +4041,7 @@
     </row>
     <row r="45">
       <c r="A45" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B45" s="5">
         <v>600000.0</v>
@@ -4107,7 +4086,7 @@
     </row>
     <row r="46">
       <c r="A46" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B46" s="5">
         <v>1216666.67</v>
@@ -4152,7 +4131,7 @@
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B47" s="5">
         <v>608333.33</v>
@@ -4197,7 +4176,7 @@
     </row>
     <row r="48">
       <c r="A48" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B48" s="7">
         <f t="shared" ref="B48:N48" si="8">SUM(B41:B47)</f>
@@ -4252,12 +4231,24 @@
         <v>73248781</v>
       </c>
     </row>
+    <row r="52">
+      <c r="I52" s="8">
+        <f>SUM(B48:G48)</f>
+        <v>32546372</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="I53" s="9">
+        <f>(N36/I52)-1</f>
+        <v>-0.7860848208</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A14:N14"/>
     <mergeCell ref="A27:N27"/>
     <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A14:N14"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>